<commit_message>
used consolidate, merge and find and replace function in excel
</commit_message>
<xml_diff>
--- a/EXCEL/Duplicate,Consolidate.xlsx
+++ b/EXCEL/Duplicate,Consolidate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="13_ncr:1_{3CD16032-BB93-41F3-AAA5-8482313C074C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03C324E2-623E-48D1-A44F-C5BDC74BF494}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:1_{3CD16032-BB93-41F3-AAA5-8482313C074C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46160EEB-E9B7-4156-8556-41585CE791B3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{B512393C-A169-4FEB-9B8A-D23DF8461FEC}"/>
+    <workbookView minimized="1" xWindow="168" yWindow="0" windowWidth="17280" windowHeight="10500" xr2:uid="{B512393C-A169-4FEB-9B8A-D23DF8461FEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <si>
     <t>StudentID</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>Malhotra</t>
+  </si>
+  <si>
+    <t>merge</t>
   </si>
 </sst>
 </file>
@@ -187,7 +190,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -198,6 +201,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -214,6 +218,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -533,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA45628F-9C24-4EB4-9E19-59CFAC2B2DE9}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="8.85546875" customWidth="1"/>
@@ -541,9 +549,10 @@
     <col min="3" max="3" width="13.85546875" customWidth="1"/>
     <col min="4" max="4" width="15.0703125" customWidth="1"/>
     <col min="5" max="5" width="31.92578125" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="42" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="42" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -565,8 +574,11 @@
       <c r="G1" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="H1" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" s="3">
         <v>101</v>
       </c>
@@ -588,8 +600,12 @@
       <c r="G2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="H2" t="str">
+        <f>F2&amp;" "&amp;G2</f>
+        <v>Raj Kumar</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" s="3">
         <v>102</v>
       </c>
@@ -611,8 +627,12 @@
       <c r="G3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="H3" t="str">
+        <f t="shared" ref="H3:H7" si="0">F3&amp;" "&amp;G3</f>
+        <v>Meena Singh</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" s="3">
         <v>104</v>
       </c>
@@ -634,8 +654,12 @@
       <c r="G4" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="H4" t="str">
+        <f t="shared" si="0"/>
+        <v>Aditi Sharma</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="3">
         <v>106</v>
       </c>
@@ -657,8 +681,12 @@
       <c r="G5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="H5" t="str">
+        <f t="shared" si="0"/>
+        <v>Soniac Sharma</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" s="3">
         <v>107</v>
       </c>
@@ -680,8 +708,12 @@
       <c r="G6" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="H6" t="str">
+        <f t="shared" si="0"/>
+        <v>Karan Gupta</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7" s="3">
         <v>108</v>
       </c>
@@ -703,8 +735,57 @@
       <c r="G7" t="s">
         <v>32</v>
       </c>
+      <c r="H7" t="str">
+        <f t="shared" si="0"/>
+        <v>Pooja Malhotra</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A10" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>7000</v>
+      </c>
     </row>
   </sheetData>
+  <dataConsolidate leftLabels="1" topLabels="1">
+    <dataRefs count="1">
+      <dataRef ref="C1:D6" sheet="Sheet1"/>
+    </dataRefs>
+  </dataConsolidate>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" display="mailto:raj.kumar@gmail.com" xr:uid="{F9BE725D-9F4D-4B8E-935E-2F2664954A32}"/>
     <hyperlink ref="E5" r:id="rId2" display="mailto:sonia123@yahoo.com" xr:uid="{C701AA3E-A4A6-4B63-AFDC-E991F81744A6}"/>

</xml_diff>